<commit_message>
21.06 New struktur of allow_codes with description and direct change and save of exel
</commit_message>
<xml_diff>
--- a/backend/testfiles/auslaender_liste.xlsx
+++ b/backend/testfiles/auslaender_liste.xlsx
@@ -14,22 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
-  <si>
-    <t>Geschlecht</t>
-  </si>
-  <si>
-    <t>Staatsangehoerigkeit</t>
-  </si>
-  <si>
-    <t>Geburtsdatum</t>
-  </si>
-  <si>
-    <t>AZR_Nummer</t>
-  </si>
-  <si>
-    <t>männlich</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>1995-08-12</t>
   </si>
@@ -49,9 +34,6 @@
     <t>12345</t>
   </si>
   <si>
-    <t>weiblich</t>
-  </si>
-  <si>
     <t>RUSSIA</t>
   </si>
   <si>
@@ -70,7 +52,22 @@
     <t>111122223333</t>
   </si>
   <si>
-    <t>01</t>
+    <t>azrNummer</t>
+  </si>
+  <si>
+    <t>geburtsdatum</t>
+  </si>
+  <si>
+    <t>geschlecht</t>
+  </si>
+  <si>
+    <t>m</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>staatsangehoerigkeit</t>
   </si>
 </sst>
 </file>
@@ -434,74 +431,77 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="14"/>
   <cols>
-    <col min="2" max="2" width="33.5" customWidth="1"/>
+    <col min="1" max="1" width="32.8984375" customWidth="1"/>
+    <col min="2" max="2" width="51.5" customWidth="1"/>
+    <col min="3" max="3" width="31.3984375" customWidth="1"/>
+    <col min="4" max="4" width="33.296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="B2" s="2">
+        <v>423</v>
       </c>
       <c r="C2" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="B5" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>